<commit_message>
feat: publish readable report 2.5 and native Sheets guidance
</commit_message>
<xml_diff>
--- a/dist/plugins/blend-kit/skills/blend-automation-test/_kit/skills/blend-generate-test-spec/assets/test-report-block-template.ja.xlsx
+++ b/dist/plugins/blend-kit/skills/blend-automation-test/_kit/skills/blend-generate-test-spec/assets/test-report-block-template.ja.xlsx
@@ -1,29 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-2025" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="概要" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="テストケース" sheetId="2" state="visible" r:id="rId2"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'概要'!$A$29:$C$30</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'概要'!$A$1:$C$30</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'テストケース'!$A$1:$F$93</definedName>
-  </definedNames>
-  <calcPr calcId="181029" fullCalcOnLoad="1"/>
-</workbook>
+<s:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <s:workbookPr filterPrivacy="1"/>
+  <s:bookViews>
+    <s:workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-2025" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </s:bookViews>
+  <s:sheets>
+    <s:sheet name="概要" sheetId="1" state="visible" r:id="rId1"/>
+    <s:sheet name="テストケース" sheetId="2" state="visible" r:id="rId2"/>
+  </s:sheets>
+  <s:definedNames>
+    <s:definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'概要'!$A$29:$C$30</s:definedName>
+    <s:definedName name="_xlnm.Print_Area" localSheetId="0">'概要'!$A$1:$C$30</s:definedName>
+    <s:definedName name="_xlnm.Print_Area" localSheetId="1">'テストケース'!$A$1:$E$13</s:definedName>
+  </s:definedNames>
+  <s:calcPr calcId="181029" fullCalcOnLoad="1"/>
+</s:workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="&quot;&#10;&quot;General;&quot;&#10;&quot;-General;&quot;&#10;&quot;General;&quot;&#10;&quot;@"/>
+    <numFmt numFmtId="166" formatCode="&quot;&#10;&quot;#,##0;&quot;&#10;&quot;-#,##0;&quot;&#10;&quot;#,##0;&quot;&#10;&quot;@"/>
+    <numFmt numFmtId="167" formatCode="&quot;&#10;&quot;0.0%;&quot;&#10;&quot;-0.0%;&quot;&#10;&quot;0.0%;&quot;&#10;&quot;@"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -101,8 +104,14 @@
       <color rgb="00172033"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -144,6 +153,11 @@
         <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017324D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -269,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -478,6 +492,94 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="8" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -764,100 +866,102 @@
   </cols>
   <sheetData>
     <row r="1" ht="32.1" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>テスト結果報告書</t>
         </is>
       </c>
-      <c r="B1" s="10" t="n"/>
+      <c r="B1" s="91" t="n"/>
+      <c r="C1" s="92" t="n"/>
     </row>
     <row r="2" ht="12" customHeight="1">
       <c r="A2" s="10" t="inlineStr"/>
       <c r="B2" s="10" t="n"/>
     </row>
     <row r="3" ht="32.1" customHeight="1">
-      <c r="A3" s="26" t="inlineStr">
+      <c r="A3" s="93" t="inlineStr">
         <is>
           <t>実行ID、アプリケーション版、環境、実施者、実施日時を入力します。</t>
         </is>
       </c>
+      <c r="C3" s="92" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="94" t="inlineStr">
         <is>
           <t>機能</t>
         </is>
       </c>
-      <c r="B4" s="49" t="inlineStr">
+      <c r="B4" s="95" t="inlineStr">
         <is>
           <t>SYN-SC synthetic rule lifecycle</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="94" t="inlineStr">
         <is>
           <t>テスト設計版</t>
         </is>
       </c>
-      <c r="B5" s="49" t="inlineStr">
+      <c r="B5" s="95" t="inlineStr">
         <is>
           <t>compact-r1</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="94" t="inlineStr">
         <is>
           <t>テスト実行ID</t>
         </is>
       </c>
-      <c r="B6" s="50" t="inlineStr"/>
+      <c r="B6" s="96" t="inlineStr"/>
       <c r="C6" s="64" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="94" t="inlineStr">
         <is>
           <t>アプリケーション版</t>
         </is>
       </c>
-      <c r="B7" s="50" t="inlineStr"/>
+      <c r="B7" s="96" t="inlineStr"/>
       <c r="C7" s="64" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="94" t="inlineStr">
         <is>
           <t>環境</t>
         </is>
       </c>
-      <c r="B8" s="50" t="inlineStr"/>
+      <c r="B8" s="96" t="inlineStr"/>
       <c r="C8" s="64" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="94" t="inlineStr">
         <is>
           <t>実施者</t>
         </is>
       </c>
-      <c r="B9" s="50" t="inlineStr"/>
+      <c r="B9" s="96" t="inlineStr"/>
       <c r="C9" s="64" t="n"/>
     </row>
     <row r="10" ht="44" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="94" t="inlineStr">
         <is>
           <t>実施日時（タイムゾーン付き）</t>
         </is>
       </c>
-      <c r="B10" s="50" t="inlineStr"/>
+      <c r="B10" s="96" t="inlineStr"/>
       <c r="C10" s="64" t="n"/>
     </row>
     <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="94" t="inlineStr">
         <is>
           <t>対象範囲</t>
         </is>
       </c>
-      <c r="B11" s="49" t="inlineStr">
+      <c r="B11" s="95" t="inlineStr">
         <is>
           <t>SYN:O1–O8; boundary, deletion, incomplete/stale rule, AND controls
 準備: TD-SC create/verify/reset once per variant; G-PREP retains unknown entry/readback seams
@@ -867,24 +971,24 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="94" t="inlineStr">
         <is>
           <t>対象外</t>
         </is>
       </c>
-      <c r="B12" s="49" t="inlineStr">
+      <c r="B12" s="95" t="inlineStr">
         <is>
           <t>八義務の除外なし。実BLEND QAはsynthetic fixture対象外。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="61" customHeight="1">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="94" t="inlineStr">
         <is>
           <t>制限事項</t>
         </is>
       </c>
-      <c r="B13" s="49" t="inlineStr">
+      <c r="B13" s="95" t="inlineStr">
         <is>
           <t>G-PREP: concrete browser/request seams are not verified
 1件の未完了事項を対応するテストケースの準備に記載しています。
@@ -897,161 +1001,174 @@
       <c r="B14" s="49" t="inlineStr"/>
     </row>
     <row r="15" ht="32.1" customHeight="1">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" s="97" t="inlineStr">
         <is>
           <t>進捗と結果</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n"/>
+      <c r="B15" s="97" t="n"/>
+      <c r="C15" s="92" t="n"/>
     </row>
     <row r="16" ht="32.1" customHeight="1">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="91" t="inlineStr">
         <is>
           <t>ケース数</t>
         </is>
       </c>
-      <c r="B16" s="51">
+      <c r="B16" s="98">
         <f>1</f>
         <v/>
       </c>
+      <c r="C16" s="92" t="n"/>
     </row>
     <row r="17" ht="32.1" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="91" t="inlineStr">
         <is>
           <t>バリエーション数</t>
         </is>
       </c>
-      <c r="B17" s="51">
+      <c r="B17" s="98">
         <f>2</f>
         <v/>
       </c>
+      <c r="C17" s="92" t="n"/>
     </row>
     <row r="18" ht="44" customHeight="1">
-      <c r="A18" s="49" t="inlineStr">
+      <c r="A18" s="95" t="inlineStr">
         <is>
           <t>対象条件を満たす合格ケース数</t>
         </is>
       </c>
-      <c r="B18" s="51">
+      <c r="B18" s="98">
         <f>COUNTIF(C30:C30,"合格")</f>
         <v/>
       </c>
+      <c r="C18" s="92" t="n"/>
     </row>
     <row r="19" ht="44" customHeight="1">
-      <c r="A19" s="49" t="inlineStr">
+      <c r="A19" s="95" t="inlineStr">
         <is>
           <t>対象条件を満たす不合格ケース数</t>
         </is>
       </c>
-      <c r="B19" s="51">
+      <c r="B19" s="98">
         <f>COUNTIF(C30:C30,"不合格")</f>
         <v/>
       </c>
+      <c r="C19" s="92" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="49" t="inlineStr">
+      <c r="A20" s="95" t="inlineStr">
         <is>
           <t>実行不可バリエーション数</t>
         </is>
       </c>
-      <c r="B20" s="51">
+      <c r="B20" s="98">
         <f>SUM('テストケース'!B90)</f>
         <v/>
       </c>
+      <c r="C20" s="92" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="49" t="inlineStr">
+      <c r="A21" s="95" t="inlineStr">
         <is>
           <t>実行省略バリエーション数</t>
         </is>
       </c>
-      <c r="B21" s="51">
+      <c r="B21" s="98">
         <f>SUM('テストケース'!B91)</f>
         <v/>
       </c>
+      <c r="C21" s="92" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="49" t="inlineStr">
+      <c r="A22" s="95" t="inlineStr">
         <is>
           <t>未実行バリエーション数</t>
         </is>
       </c>
-      <c r="B22" s="51">
+      <c r="B22" s="98">
         <f>SUM('テストケース'!B92)</f>
         <v/>
       </c>
+      <c r="C22" s="92" t="n"/>
     </row>
     <row r="23" ht="44" customHeight="1">
-      <c r="A23" s="49" t="inlineStr">
+      <c r="A23" s="95" t="inlineStr">
         <is>
           <t>対象条件を満たす合否判定ケース数</t>
         </is>
       </c>
-      <c r="B23" s="51">
+      <c r="B23" s="98">
         <f>B18+B19</f>
         <v/>
       </c>
+      <c r="C23" s="92" t="n"/>
     </row>
     <row r="24" ht="44" customHeight="1">
-      <c r="A24" s="49" t="inlineStr">
+      <c r="A24" s="95" t="inlineStr">
         <is>
           <t>合格ケース数 / 対象条件を満たす合否判定ケース数</t>
         </is>
       </c>
-      <c r="B24" s="52">
+      <c r="B24" s="99">
         <f>IF(B23=0,"データなし",B18/B23)</f>
         <v/>
       </c>
+      <c r="C24" s="92" t="n"/>
     </row>
     <row r="25" ht="44" customHeight="1">
-      <c r="A25" s="49" t="inlineStr">
+      <c r="A25" s="95" t="inlineStr">
         <is>
           <t>対象条件を満たす合否判定ケース数 / 全ケース数</t>
         </is>
       </c>
-      <c r="B25" s="52">
+      <c r="B25" s="99">
         <f>IF(B16=0,"データなし",B23/B16)</f>
         <v/>
       </c>
+      <c r="C25" s="92" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="49" t="inlineStr">
+      <c r="A26" s="95" t="inlineStr">
         <is>
           <t>合格未確認ケース数</t>
         </is>
       </c>
-      <c r="B26" s="51">
+      <c r="B26" s="98">
         <f>B16-B18</f>
         <v/>
       </c>
+      <c r="C26" s="92" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="49" t="inlineStr">
+      <c r="A27" s="95" t="inlineStr">
         <is>
           <t>無効なバリエーション状態数</t>
         </is>
       </c>
-      <c r="B27" s="51">
+      <c r="B27" s="98">
         <f>B17-SUM(B20:B22,SUM('テストケース'!B88),SUM('テストケース'!B89))</f>
         <v/>
       </c>
+      <c r="C27" s="92" t="n"/>
     </row>
     <row r="28" ht="32.1" customHeight="1">
       <c r="A28" s="10" t="n"/>
       <c r="B28" s="10" t="n"/>
     </row>
     <row r="29" ht="32.1" customHeight="1">
-      <c r="A29" s="30" t="inlineStr">
+      <c r="A29" s="97" t="inlineStr">
         <is>
           <t>テストID</t>
         </is>
       </c>
-      <c r="B29" s="30" t="inlineStr">
+      <c r="B29" s="97" t="inlineStr">
         <is>
           <t>テストケース</t>
         </is>
       </c>
-      <c r="C29" s="30" t="inlineStr">
+      <c r="C29" s="97" t="inlineStr">
         <is>
           <t>集計状態</t>
         </is>
@@ -1086,59 +1203,174 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="5"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="5"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32.1" customHeight="1">
-      <c r="A1" s="70" t="inlineStr">
+      <c r="A1" s="100" t="inlineStr">
         <is>
           <t>テストケース詳細</t>
         </is>
       </c>
-      <c r="B1" s="71" t="n"/>
-      <c r="C1" s="71" t="n"/>
-      <c r="D1" s="71" t="n"/>
-      <c r="E1" s="71" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1">
+      <c r="B1" s="92" t="n"/>
+      <c r="C1" s="92" t="n"/>
+      <c r="D1" s="92" t="n"/>
+      <c r="E1" s="92" t="n"/>
+    </row>
+    <row r="2" hidden="1" ht="42" customHeight="1">
       <c r="A2" s="72" t="inlineStr"/>
-      <c r="B2" s="71" t="n"/>
-      <c r="C2" s="71" t="n"/>
-      <c r="D2" s="71" t="n"/>
-      <c r="E2" s="71" t="n"/>
-    </row>
-    <row r="3" ht="12" customHeight="1">
+    </row>
+    <row r="3" hidden="1" ht="12" customHeight="1">
       <c r="A3" s="71" t="n"/>
       <c r="B3" s="71" t="n"/>
       <c r="C3" s="71" t="n"/>
       <c r="D3" s="71" t="n"/>
       <c r="E3" s="71" t="n"/>
     </row>
-    <row r="4" ht="8" customHeight="1">
+    <row r="4" hidden="1" ht="8" customHeight="1">
       <c r="A4" s="73" t="n"/>
       <c r="B4" s="71" t="n"/>
       <c r="C4" s="71" t="n"/>
       <c r="D4" s="71" t="n"/>
       <c r="E4" s="71" t="n"/>
     </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="101" t="inlineStr">
+        <is>
+          <t>[テストID] — [ケース名]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="95" t="inlineStr">
+        <is>
+          <t>ケース結果</t>
+        </is>
+      </c>
+      <c r="B6" s="95" t="inlineStr">
+        <is>
+          <t>未実行</t>
+        </is>
+      </c>
+      <c r="C6" s="92" t="n"/>
+      <c r="D6" s="92" t="n"/>
+      <c r="E6" s="92" t="n"/>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="95" t="inlineStr">
+        <is>
+          <t>前提</t>
+        </is>
+      </c>
+      <c r="B7" s="95" t="inlineStr">
+        <is>
+          <t>[初期状態と共通データ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="95" t="inlineStr">
+        <is>
+          <t>ステップ</t>
+        </is>
+      </c>
+      <c r="B8" s="95" t="inlineStr">
+        <is>
+          <t>共通操作</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="95" t="inlineStr">
+        <is>
+          <t>ステップ 1</t>
+        </is>
+      </c>
+      <c r="B9" s="95" t="inlineStr">
+        <is>
+          <t>[共通の操作]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>条件</t>
+        </is>
+      </c>
+      <c r="B10" s="73" t="inlineStr">
+        <is>
+          <t>データ・個別操作</t>
+        </is>
+      </c>
+      <c r="C10" s="73" t="inlineStr">
+        <is>
+          <t>期待結果</t>
+        </is>
+      </c>
+      <c r="D10" s="73" t="inlineStr">
+        <is>
+          <t>実際の結果</t>
+        </is>
+      </c>
+      <c r="E10" s="73" t="inlineStr">
+        <is>
+          <t>結果</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="3" customHeight="1">
+      <c r="D11" s="29" t="n"/>
+      <c r="E11" s="29" t="n"/>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>削除を取り消す (cancel)</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>確認画面でキャンセルを選択。</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>ルールは2件とも維持。</t>
+        </is>
+      </c>
+      <c r="D12" s="102" t="inlineStr"/>
+      <c r="E12" s="102" t="inlineStr">
+        <is>
+          <t>未実行</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="95" t="inlineStr">
+        <is>
+          <t>証拠画像 — 画像なし</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="6">
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B8:E8"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A13:E13"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="E15 E16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
-      <formula1>"合格,不合格,実行不可,実行省略,未実行"</formula1>
-    </dataValidation>
-  </dataValidations>
   <printOptions horizontalCentered="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="8" fitToHeight="0" fitToWidth="1"/>

</xml_diff>